<commit_message>
2026 06 03 modification du débit
</commit_message>
<xml_diff>
--- a/modeles_excel/V3.01_modèle_final.xlsx
+++ b/modeles_excel/V3.01_modèle_final.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10412"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10525"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/souchaud/Documents/Travail/CitizenSers/Spectroscopie/traitement_données/spectroscopie_raman/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/souchaud/Documents/Travail/CitizenSers/02_Spectroscopie/traitement_données/spectroscopie_raman/modeles_excel/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9543639D-8D5A-B245-8249-284DF8B83B0D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A4E1FB3A-E2C3-D840-8FF0-F6DDC341FABA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-38300" yWindow="-7780" windowWidth="37860" windowHeight="24960" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,7 +16,7 @@
     <sheet name="Mesures" sheetId="1" r:id="rId1"/>
     <sheet name="Listes" sheetId="2" r:id="rId2"/>
   </sheets>
-  <calcPr calcId="191029" iterateDelta="1E-4"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="95" uniqueCount="76">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="90" uniqueCount="71">
   <si>
     <t>Dispositif de mesure de la qualité de l'eau par les citoyens</t>
   </si>
@@ -194,27 +194,6 @@
     <t>Lieu de la titration</t>
   </si>
   <si>
-    <t>Débit / flux</t>
-  </si>
-  <si>
-    <t>Débit / flux - Largeur route</t>
-  </si>
-  <si>
-    <t>Débit / flux - Longueur 6 arches</t>
-  </si>
-  <si>
-    <t>Débit / flux - Hauteur eau</t>
-  </si>
-  <si>
-    <t>Débit / flux - Volume total (m3)</t>
-  </si>
-  <si>
-    <t>Débit / flux - Vitesse (s)</t>
-  </si>
-  <si>
-    <t>Débit / flux - Débit (m3/s)</t>
-  </si>
-  <si>
     <t>Commentaires</t>
   </si>
   <si>
@@ -261,6 +240,12 @@
   </si>
   <si>
     <t xml:space="preserve">Coordinateur·ice : </t>
+  </si>
+  <si>
+    <t>Débit</t>
+  </si>
+  <si>
+    <t>Débit (m3/s)</t>
   </si>
 </sst>
 </file>
@@ -428,12 +413,6 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFB58FBD"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor theme="5" tint="0.59999389629810485"/>
         <bgColor indexed="64"/>
       </patternFill>
@@ -448,6 +427,11 @@
       <patternFill patternType="solid">
         <fgColor theme="6" tint="0.59999389629810485"/>
         <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFF2CC"/>
       </patternFill>
     </fill>
   </fills>
@@ -746,7 +730,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5"/>
   </cellStyleXfs>
-  <cellXfs count="97">
+  <cellXfs count="99">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyProtection="1">
       <protection locked="0"/>
@@ -862,31 +846,31 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="19" borderId="18" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="19" borderId="19" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="19" borderId="14" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="19" borderId="15" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="19" borderId="20" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="19" borderId="21" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="19" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="0" fillId="18" borderId="18" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="18" borderId="19" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="18" borderId="14" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="18" borderId="15" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="18" borderId="20" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="18" borderId="21" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="18" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
@@ -896,7 +880,7 @@
     <xf numFmtId="0" fontId="2" fillId="4" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="20" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="19" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -906,9 +890,6 @@
     <xf numFmtId="0" fontId="2" fillId="16" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="6" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -927,7 +908,7 @@
     <xf numFmtId="0" fontId="2" fillId="5" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="18" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="17" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
@@ -981,15 +962,15 @@
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="19" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="4" fillId="18" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="19" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="4" fillId="18" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="19" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="4" fillId="18" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
     </xf>
@@ -997,15 +978,15 @@
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="19" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="4" fillId="18" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="19" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="4" fillId="18" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="19" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="4" fillId="18" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
     </xf>
@@ -1016,12 +997,15 @@
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="17" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="17" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="25" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyProtection="1">
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -1034,22 +1018,19 @@
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1" applyProtection="1">
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1" applyProtection="1">
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="14" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="17" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1" applyProtection="1">
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1" applyProtection="1">
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="14" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="18" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1081,15 +1062,25 @@
     <xf numFmtId="0" fontId="3" fillId="16" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="25" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyProtection="1">
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="20" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="20" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1442,42 +1433,42 @@
       <c r="F1" s="77"/>
       <c r="G1" s="77"/>
       <c r="H1" s="78"/>
-      <c r="I1" s="54"/>
-      <c r="L1" s="51"/>
-      <c r="M1" s="52"/>
-      <c r="N1" s="52"/>
-      <c r="O1" s="52"/>
-      <c r="P1" s="52"/>
-      <c r="Q1" s="52"/>
-      <c r="R1" s="52"/>
-      <c r="S1" s="52"/>
+      <c r="I1" s="53"/>
+      <c r="L1" s="50"/>
+      <c r="M1" s="51"/>
+      <c r="N1" s="51"/>
+      <c r="O1" s="51"/>
+      <c r="P1" s="51"/>
+      <c r="Q1" s="51"/>
+      <c r="R1" s="51"/>
+      <c r="S1" s="51"/>
     </row>
     <row r="2" spans="1:19" ht="22" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="85" t="s">
+      <c r="A2" s="84" t="s">
         <v>1</v>
       </c>
       <c r="B2" s="77"/>
       <c r="C2" s="77"/>
       <c r="D2" s="77"/>
-      <c r="E2" s="86"/>
-      <c r="F2" s="86"/>
-      <c r="G2" s="86"/>
-      <c r="H2" s="87"/>
-      <c r="I2" s="54"/>
-      <c r="L2" s="51"/>
-      <c r="M2" s="52"/>
-      <c r="N2" s="52"/>
-      <c r="O2" s="52"/>
-      <c r="P2" s="52"/>
-      <c r="Q2" s="52"/>
-      <c r="R2" s="52"/>
-      <c r="S2" s="52"/>
+      <c r="E2" s="85"/>
+      <c r="F2" s="85"/>
+      <c r="G2" s="85"/>
+      <c r="H2" s="86"/>
+      <c r="I2" s="53"/>
+      <c r="L2" s="50"/>
+      <c r="M2" s="51"/>
+      <c r="N2" s="51"/>
+      <c r="O2" s="51"/>
+      <c r="P2" s="51"/>
+      <c r="Q2" s="51"/>
+      <c r="R2" s="51"/>
+      <c r="S2" s="51"/>
     </row>
     <row r="3" spans="1:19" ht="39" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="37" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="72" t="str">
+      <c r="B3" s="71" t="str">
         <f>IF(OR(B8="",B9="",B5="",D5=""),"","PRE_"&amp;UPPER(LEFT(B8,1))&amp;UPPER(MID(B8,FIND(" ",B8&amp;" ")+1,1))&amp;UPPER(LEFT(B9,1))&amp;UPPER(MID(B9,FIND(" ",B9&amp;" ")+1,1))&amp;"_"&amp;TEXT(B5,"aaaammjj")&amp;"_"&amp;TEXT(D5,"hh\hmm"))</f>
         <v/>
       </c>
@@ -1489,15 +1480,15 @@
       <c r="F3" s="32"/>
       <c r="G3" s="32"/>
       <c r="H3" s="33"/>
-      <c r="I3" s="54"/>
-      <c r="L3" s="53"/>
-      <c r="M3" s="54"/>
-      <c r="N3" s="53"/>
-      <c r="O3" s="54"/>
-      <c r="P3" s="54"/>
-      <c r="Q3" s="54"/>
-      <c r="R3" s="54"/>
-      <c r="S3" s="54"/>
+      <c r="I3" s="53"/>
+      <c r="L3" s="52"/>
+      <c r="M3" s="53"/>
+      <c r="N3" s="52"/>
+      <c r="O3" s="53"/>
+      <c r="P3" s="53"/>
+      <c r="Q3" s="53"/>
+      <c r="R3" s="53"/>
+      <c r="S3" s="53"/>
     </row>
     <row r="4" spans="1:19" ht="22" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="37" t="s">
@@ -1512,15 +1503,15 @@
       <c r="F4" s="30"/>
       <c r="G4" s="30"/>
       <c r="H4" s="35"/>
-      <c r="I4" s="54"/>
-      <c r="L4" s="53"/>
-      <c r="M4" s="54"/>
-      <c r="N4" s="63"/>
-      <c r="O4" s="54"/>
-      <c r="P4" s="54"/>
-      <c r="Q4" s="54"/>
-      <c r="R4" s="54"/>
-      <c r="S4" s="54"/>
+      <c r="I4" s="53"/>
+      <c r="L4" s="52"/>
+      <c r="M4" s="53"/>
+      <c r="N4" s="62"/>
+      <c r="O4" s="53"/>
+      <c r="P4" s="53"/>
+      <c r="Q4" s="53"/>
+      <c r="R4" s="53"/>
+      <c r="S4" s="53"/>
     </row>
     <row r="5" spans="1:19" ht="22" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="37" t="s">
@@ -1535,15 +1526,15 @@
       <c r="F5" s="30"/>
       <c r="G5" s="30"/>
       <c r="H5" s="35"/>
-      <c r="I5" s="54"/>
-      <c r="L5" s="53"/>
-      <c r="M5" s="54"/>
-      <c r="N5" s="53"/>
-      <c r="O5" s="54"/>
-      <c r="P5" s="53"/>
-      <c r="Q5" s="54"/>
-      <c r="R5" s="54"/>
-      <c r="S5" s="54"/>
+      <c r="I5" s="53"/>
+      <c r="L5" s="52"/>
+      <c r="M5" s="53"/>
+      <c r="N5" s="52"/>
+      <c r="O5" s="53"/>
+      <c r="P5" s="52"/>
+      <c r="Q5" s="53"/>
+      <c r="R5" s="53"/>
+      <c r="S5" s="53"/>
     </row>
     <row r="6" spans="1:19" ht="54" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="37" t="s">
@@ -1558,15 +1549,15 @@
       <c r="F6" s="30"/>
       <c r="G6" s="30"/>
       <c r="H6" s="35"/>
-      <c r="I6" s="54"/>
-      <c r="L6" s="53"/>
-      <c r="M6" s="55"/>
-      <c r="N6" s="53"/>
-      <c r="O6" s="56"/>
-      <c r="P6" s="54"/>
-      <c r="Q6" s="54"/>
-      <c r="R6" s="54"/>
-      <c r="S6" s="54"/>
+      <c r="I6" s="53"/>
+      <c r="L6" s="52"/>
+      <c r="M6" s="54"/>
+      <c r="N6" s="52"/>
+      <c r="O6" s="55"/>
+      <c r="P6" s="53"/>
+      <c r="Q6" s="53"/>
+      <c r="R6" s="53"/>
+      <c r="S6" s="53"/>
     </row>
     <row r="7" spans="1:19" ht="22" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="37" t="s">
@@ -1581,15 +1572,15 @@
       <c r="F7" s="30"/>
       <c r="G7" s="30"/>
       <c r="H7" s="35"/>
-      <c r="I7" s="54"/>
-      <c r="L7" s="53"/>
-      <c r="M7" s="54"/>
-      <c r="N7" s="53"/>
-      <c r="O7" s="54"/>
-      <c r="P7" s="54"/>
-      <c r="Q7" s="54"/>
-      <c r="R7" s="54"/>
-      <c r="S7" s="54"/>
+      <c r="I7" s="53"/>
+      <c r="L7" s="52"/>
+      <c r="M7" s="53"/>
+      <c r="N7" s="52"/>
+      <c r="O7" s="53"/>
+      <c r="P7" s="53"/>
+      <c r="Q7" s="53"/>
+      <c r="R7" s="53"/>
+      <c r="S7" s="53"/>
     </row>
     <row r="8" spans="1:19" ht="22" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="37" t="s">
@@ -1604,115 +1595,115 @@
       <c r="F8" s="30"/>
       <c r="G8" s="30"/>
       <c r="H8" s="35"/>
-      <c r="I8" s="54"/>
-      <c r="L8" s="53"/>
-      <c r="M8" s="54"/>
-      <c r="N8" s="53"/>
-      <c r="O8" s="54"/>
-      <c r="P8" s="54"/>
-      <c r="Q8" s="54"/>
-      <c r="R8" s="54"/>
-      <c r="S8" s="54"/>
+      <c r="I8" s="53"/>
+      <c r="L8" s="52"/>
+      <c r="M8" s="53"/>
+      <c r="N8" s="52"/>
+      <c r="O8" s="53"/>
+      <c r="P8" s="53"/>
+      <c r="Q8" s="53"/>
+      <c r="R8" s="53"/>
+      <c r="S8" s="53"/>
     </row>
     <row r="9" spans="1:19" ht="21" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9" s="38" t="s">
         <v>14</v>
       </c>
-      <c r="B9" s="64"/>
+      <c r="B9" s="63"/>
       <c r="C9" s="8" t="s">
         <v>13</v>
       </c>
-      <c r="D9" s="64"/>
-      <c r="E9" s="65"/>
-      <c r="F9" s="66"/>
-      <c r="G9" s="66"/>
-      <c r="H9" s="67"/>
-      <c r="I9" s="68"/>
-      <c r="J9" s="57"/>
-      <c r="K9" s="57"/>
-      <c r="L9" s="57"/>
-      <c r="M9" s="57"/>
-      <c r="N9" s="57"/>
-      <c r="O9" s="57"/>
-      <c r="P9" s="57"/>
-      <c r="Q9" s="57"/>
-      <c r="R9" s="57"/>
-      <c r="S9" s="57"/>
+      <c r="D9" s="63"/>
+      <c r="E9" s="64"/>
+      <c r="F9" s="65"/>
+      <c r="G9" s="65"/>
+      <c r="H9" s="66"/>
+      <c r="I9" s="67"/>
+      <c r="J9" s="56"/>
+      <c r="K9" s="56"/>
+      <c r="L9" s="56"/>
+      <c r="M9" s="56"/>
+      <c r="N9" s="56"/>
+      <c r="O9" s="56"/>
+      <c r="P9" s="56"/>
+      <c r="Q9" s="56"/>
+      <c r="R9" s="56"/>
+      <c r="S9" s="56"/>
     </row>
     <row r="10" spans="1:19" ht="23" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="38" t="s">
         <v>15</v>
       </c>
-      <c r="B10" s="64"/>
+      <c r="B10" s="63"/>
       <c r="C10" s="8" t="s">
         <v>13</v>
       </c>
-      <c r="D10" s="64"/>
-      <c r="E10" s="65"/>
-      <c r="F10" s="66"/>
-      <c r="G10" s="66"/>
-      <c r="H10" s="67"/>
-      <c r="I10" s="68"/>
-      <c r="J10" s="57"/>
-      <c r="K10" s="57"/>
-      <c r="L10" s="57"/>
-      <c r="M10" s="57"/>
-      <c r="N10" s="57"/>
-      <c r="O10" s="57"/>
-      <c r="P10" s="57"/>
-      <c r="Q10" s="57"/>
-      <c r="R10" s="57"/>
-      <c r="S10" s="57"/>
+      <c r="D10" s="63"/>
+      <c r="E10" s="64"/>
+      <c r="F10" s="65"/>
+      <c r="G10" s="65"/>
+      <c r="H10" s="66"/>
+      <c r="I10" s="67"/>
+      <c r="J10" s="56"/>
+      <c r="K10" s="56"/>
+      <c r="L10" s="56"/>
+      <c r="M10" s="56"/>
+      <c r="N10" s="56"/>
+      <c r="O10" s="56"/>
+      <c r="P10" s="56"/>
+      <c r="Q10" s="56"/>
+      <c r="R10" s="56"/>
+      <c r="S10" s="56"/>
     </row>
     <row r="11" spans="1:19" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A11" s="38" t="s">
         <v>16</v>
       </c>
-      <c r="B11" s="64"/>
+      <c r="B11" s="63"/>
       <c r="C11" s="8" t="s">
         <v>13</v>
       </c>
-      <c r="D11" s="64"/>
-      <c r="E11" s="65"/>
-      <c r="F11" s="66"/>
-      <c r="G11" s="66"/>
-      <c r="H11" s="67"/>
-      <c r="I11" s="68"/>
-      <c r="J11" s="57"/>
-      <c r="K11" s="57"/>
-      <c r="L11" s="57"/>
-      <c r="M11" s="57"/>
-      <c r="N11" s="57"/>
-      <c r="O11" s="57"/>
-      <c r="P11" s="57"/>
-      <c r="Q11" s="57"/>
-      <c r="R11" s="57"/>
-      <c r="S11" s="57"/>
+      <c r="D11" s="63"/>
+      <c r="E11" s="64"/>
+      <c r="F11" s="65"/>
+      <c r="G11" s="65"/>
+      <c r="H11" s="66"/>
+      <c r="I11" s="67"/>
+      <c r="J11" s="56"/>
+      <c r="K11" s="56"/>
+      <c r="L11" s="56"/>
+      <c r="M11" s="56"/>
+      <c r="N11" s="56"/>
+      <c r="O11" s="56"/>
+      <c r="P11" s="56"/>
+      <c r="Q11" s="56"/>
+      <c r="R11" s="56"/>
+      <c r="S11" s="56"/>
     </row>
     <row r="12" spans="1:19" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A12" s="38" t="s">
         <v>17</v>
       </c>
-      <c r="B12" s="64"/>
+      <c r="B12" s="63"/>
       <c r="C12" s="8" t="s">
         <v>13</v>
       </c>
-      <c r="D12" s="64"/>
-      <c r="E12" s="69"/>
-      <c r="F12" s="70"/>
-      <c r="G12" s="70"/>
-      <c r="H12" s="71"/>
-      <c r="I12" s="68"/>
-      <c r="J12" s="57"/>
-      <c r="K12" s="57"/>
-      <c r="L12" s="57"/>
-      <c r="M12" s="57"/>
-      <c r="N12" s="57"/>
-      <c r="O12" s="57"/>
-      <c r="P12" s="57"/>
-      <c r="Q12" s="57"/>
-      <c r="R12" s="57"/>
-      <c r="S12" s="57"/>
+      <c r="D12" s="63"/>
+      <c r="E12" s="68"/>
+      <c r="F12" s="69"/>
+      <c r="G12" s="69"/>
+      <c r="H12" s="70"/>
+      <c r="I12" s="67"/>
+      <c r="J12" s="56"/>
+      <c r="K12" s="56"/>
+      <c r="L12" s="56"/>
+      <c r="M12" s="56"/>
+      <c r="N12" s="56"/>
+      <c r="O12" s="56"/>
+      <c r="P12" s="56"/>
+      <c r="Q12" s="56"/>
+      <c r="R12" s="56"/>
+      <c r="S12" s="56"/>
     </row>
     <row r="13" spans="1:19" ht="28" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A13" s="39" t="s">
@@ -1739,17 +1730,17 @@
       <c r="H13" s="19" t="s">
         <v>19</v>
       </c>
-      <c r="I13" s="68"/>
-      <c r="J13" s="57"/>
-      <c r="K13" s="57"/>
-      <c r="L13" s="53"/>
-      <c r="M13" s="54"/>
-      <c r="N13" s="53"/>
-      <c r="O13" s="54"/>
-      <c r="P13" s="53"/>
-      <c r="Q13" s="54"/>
-      <c r="R13" s="53"/>
-      <c r="S13" s="54"/>
+      <c r="I13" s="67"/>
+      <c r="J13" s="56"/>
+      <c r="K13" s="56"/>
+      <c r="L13" s="52"/>
+      <c r="M13" s="53"/>
+      <c r="N13" s="52"/>
+      <c r="O13" s="53"/>
+      <c r="P13" s="52"/>
+      <c r="Q13" s="53"/>
+      <c r="R13" s="52"/>
+      <c r="S13" s="53"/>
     </row>
     <row r="14" spans="1:19" ht="26" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A14" s="40" t="s">
@@ -1772,95 +1763,95 @@
       </c>
       <c r="G14" s="27"/>
       <c r="H14" s="27"/>
-      <c r="I14" s="68"/>
-      <c r="J14" s="57"/>
-      <c r="K14" s="57"/>
-      <c r="L14" s="53"/>
-      <c r="M14" s="54"/>
-      <c r="N14" s="53"/>
-      <c r="O14" s="54"/>
-      <c r="P14" s="53"/>
-      <c r="Q14" s="54"/>
-      <c r="R14" s="54"/>
-      <c r="S14" s="54"/>
+      <c r="I14" s="67"/>
+      <c r="J14" s="56"/>
+      <c r="K14" s="56"/>
+      <c r="L14" s="52"/>
+      <c r="M14" s="53"/>
+      <c r="N14" s="52"/>
+      <c r="O14" s="53"/>
+      <c r="P14" s="52"/>
+      <c r="Q14" s="53"/>
+      <c r="R14" s="53"/>
+      <c r="S14" s="53"/>
     </row>
     <row r="15" spans="1:19" ht="22" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A15"/>
-      <c r="I15" s="57"/>
-      <c r="J15" s="57"/>
-      <c r="K15" s="57"/>
-      <c r="L15" s="57"/>
-      <c r="M15" s="57"/>
-      <c r="N15" s="57"/>
-      <c r="O15" s="57"/>
-      <c r="P15" s="57"/>
-      <c r="Q15" s="57"/>
-      <c r="R15" s="57"/>
-      <c r="S15" s="57"/>
+      <c r="I15" s="56"/>
+      <c r="J15" s="56"/>
+      <c r="K15" s="56"/>
+      <c r="L15" s="56"/>
+      <c r="M15" s="56"/>
+      <c r="N15" s="56"/>
+      <c r="O15" s="56"/>
+      <c r="P15" s="56"/>
+      <c r="Q15" s="56"/>
+      <c r="R15" s="56"/>
+      <c r="S15" s="56"/>
     </row>
     <row r="16" spans="1:19" ht="22" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="88" t="s">
+      <c r="A16" s="87" t="s">
         <v>26</v>
       </c>
-      <c r="B16" s="89"/>
-      <c r="C16" s="89"/>
-      <c r="D16" s="89"/>
-      <c r="E16" s="89"/>
-      <c r="F16" s="89"/>
-      <c r="G16" s="89"/>
-      <c r="H16" s="90"/>
-      <c r="I16" s="57"/>
-      <c r="J16" s="57"/>
-      <c r="K16" s="57"/>
-      <c r="L16" s="51"/>
-      <c r="M16" s="51"/>
-      <c r="N16" s="51"/>
-      <c r="O16" s="51"/>
-      <c r="P16" s="51"/>
-      <c r="Q16" s="51"/>
-      <c r="R16" s="51"/>
-      <c r="S16" s="51"/>
+      <c r="B16" s="88"/>
+      <c r="C16" s="88"/>
+      <c r="D16" s="88"/>
+      <c r="E16" s="88"/>
+      <c r="F16" s="88"/>
+      <c r="G16" s="88"/>
+      <c r="H16" s="89"/>
+      <c r="I16" s="56"/>
+      <c r="J16" s="56"/>
+      <c r="K16" s="56"/>
+      <c r="L16" s="50"/>
+      <c r="M16" s="50"/>
+      <c r="N16" s="50"/>
+      <c r="O16" s="50"/>
+      <c r="P16" s="50"/>
+      <c r="Q16" s="50"/>
+      <c r="R16" s="50"/>
+      <c r="S16" s="50"/>
     </row>
     <row r="17" spans="1:19" ht="22" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A17"/>
-      <c r="I17" s="57"/>
-      <c r="J17" s="57"/>
-      <c r="K17" s="57"/>
-      <c r="L17" s="58"/>
-      <c r="M17" s="57"/>
-      <c r="N17" s="57"/>
-      <c r="O17" s="57"/>
-      <c r="P17" s="57"/>
-      <c r="Q17" s="57"/>
-      <c r="R17" s="57"/>
-      <c r="S17" s="57"/>
+      <c r="I17" s="56"/>
+      <c r="J17" s="56"/>
+      <c r="K17" s="56"/>
+      <c r="L17" s="57"/>
+      <c r="M17" s="56"/>
+      <c r="N17" s="56"/>
+      <c r="O17" s="56"/>
+      <c r="P17" s="56"/>
+      <c r="Q17" s="56"/>
+      <c r="R17" s="56"/>
+      <c r="S17" s="56"/>
     </row>
     <row r="18" spans="1:19" ht="22" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A18" s="93" t="s">
+      <c r="A18" s="92" t="s">
         <v>27</v>
       </c>
-      <c r="B18" s="80"/>
-      <c r="C18" s="80"/>
-      <c r="D18" s="80"/>
-      <c r="E18" s="80"/>
-      <c r="F18" s="81"/>
+      <c r="B18" s="79"/>
+      <c r="C18" s="79"/>
+      <c r="D18" s="79"/>
+      <c r="E18" s="79"/>
+      <c r="F18" s="80"/>
       <c r="G18" s="21"/>
       <c r="H18" s="21"/>
-      <c r="I18" s="57"/>
-      <c r="J18" s="57"/>
-      <c r="K18" s="57"/>
-      <c r="L18" s="53"/>
-      <c r="M18" s="53"/>
-      <c r="N18" s="53"/>
-      <c r="O18" s="53"/>
-      <c r="P18" s="53"/>
-      <c r="Q18" s="53"/>
-      <c r="R18" s="57"/>
-      <c r="S18" s="57"/>
+      <c r="I18" s="56"/>
+      <c r="J18" s="56"/>
+      <c r="K18" s="56"/>
+      <c r="L18" s="52"/>
+      <c r="M18" s="52"/>
+      <c r="N18" s="52"/>
+      <c r="O18" s="52"/>
+      <c r="P18" s="52"/>
+      <c r="Q18" s="52"/>
+      <c r="R18" s="56"/>
+      <c r="S18" s="56"/>
     </row>
     <row r="19" spans="1:19" ht="26" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A19" s="42" t="s">
-        <v>62</v>
+        <v>55</v>
       </c>
       <c r="B19" s="22" t="s">
         <v>28</v>
@@ -1879,52 +1870,52 @@
       </c>
       <c r="G19" s="21"/>
       <c r="H19" s="21"/>
-      <c r="I19" s="57"/>
-      <c r="J19" s="57"/>
-      <c r="K19" s="57"/>
-      <c r="L19" s="54"/>
-      <c r="M19" s="54"/>
-      <c r="N19" s="54"/>
-      <c r="O19" s="54"/>
-      <c r="P19" s="54"/>
-      <c r="Q19" s="54"/>
-      <c r="R19" s="57"/>
-      <c r="S19" s="57"/>
+      <c r="I19" s="56"/>
+      <c r="J19" s="56"/>
+      <c r="K19" s="56"/>
+      <c r="L19" s="53"/>
+      <c r="M19" s="53"/>
+      <c r="N19" s="53"/>
+      <c r="O19" s="53"/>
+      <c r="P19" s="53"/>
+      <c r="Q19" s="53"/>
+      <c r="R19" s="56"/>
+      <c r="S19" s="56"/>
     </row>
     <row r="20" spans="1:19" ht="22" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="94" t="s">
-        <v>72</v>
+      <c r="A20" s="73" t="s">
+        <v>65</v>
       </c>
       <c r="B20" s="12"/>
-      <c r="C20" s="95"/>
+      <c r="C20" s="74"/>
       <c r="D20" s="12"/>
       <c r="E20" s="11"/>
       <c r="F20" s="11"/>
-      <c r="I20" s="57"/>
-      <c r="J20" s="57"/>
-      <c r="K20" s="57"/>
-      <c r="L20" s="57"/>
-      <c r="M20" s="57"/>
-      <c r="N20" s="57"/>
-      <c r="O20" s="57"/>
-      <c r="P20" s="57"/>
-      <c r="Q20" s="57"/>
-      <c r="R20" s="57"/>
-      <c r="S20" s="57"/>
+      <c r="I20" s="56"/>
+      <c r="J20" s="56"/>
+      <c r="K20" s="56"/>
+      <c r="L20" s="56"/>
+      <c r="M20" s="56"/>
+      <c r="N20" s="56"/>
+      <c r="O20" s="56"/>
+      <c r="P20" s="56"/>
+      <c r="Q20" s="56"/>
+      <c r="R20" s="56"/>
+      <c r="S20" s="56"/>
     </row>
     <row r="21" spans="1:19" ht="22" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A21"/>
-      <c r="I21" s="57"/>
-      <c r="J21" s="57"/>
-      <c r="K21" s="57"/>
-      <c r="L21" s="57"/>
-      <c r="M21" s="57"/>
-      <c r="N21" s="57"/>
-      <c r="O21" s="57"/>
-      <c r="P21" s="57"/>
-      <c r="Q21" s="57"/>
-      <c r="R21" s="57"/>
-      <c r="S21" s="57"/>
+      <c r="I21" s="56"/>
+      <c r="J21" s="56"/>
+      <c r="K21" s="56"/>
+      <c r="L21" s="56"/>
+      <c r="M21" s="56"/>
+      <c r="N21" s="56"/>
+      <c r="O21" s="56"/>
+      <c r="P21" s="56"/>
+      <c r="Q21" s="56"/>
+      <c r="R21" s="56"/>
+      <c r="S21" s="56"/>
     </row>
     <row r="22" spans="1:19" ht="22" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A22"/>
@@ -1932,43 +1923,43 @@
       <c r="F22" s="21"/>
       <c r="G22" s="21"/>
       <c r="H22" s="21"/>
-      <c r="I22" s="57"/>
-      <c r="J22" s="57"/>
-      <c r="K22" s="57"/>
-      <c r="L22" s="58"/>
-      <c r="M22" s="57"/>
-      <c r="N22" s="57"/>
-      <c r="O22" s="57"/>
-      <c r="P22" s="57"/>
-      <c r="Q22" s="57"/>
-      <c r="R22" s="57"/>
-      <c r="S22" s="57"/>
+      <c r="I22" s="56"/>
+      <c r="J22" s="56"/>
+      <c r="K22" s="56"/>
+      <c r="L22" s="57"/>
+      <c r="M22" s="56"/>
+      <c r="N22" s="56"/>
+      <c r="O22" s="56"/>
+      <c r="P22" s="56"/>
+      <c r="Q22" s="56"/>
+      <c r="R22" s="56"/>
+      <c r="S22" s="56"/>
     </row>
     <row r="23" spans="1:19" ht="22" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A23" s="92" t="s">
+      <c r="A23" s="91" t="s">
         <v>33</v>
       </c>
-      <c r="B23" s="80"/>
-      <c r="C23" s="80"/>
-      <c r="D23" s="80"/>
-      <c r="E23" s="81"/>
+      <c r="B23" s="79"/>
+      <c r="C23" s="79"/>
+      <c r="D23" s="79"/>
+      <c r="E23" s="80"/>
       <c r="F23" s="21"/>
       <c r="G23" s="21"/>
       <c r="H23" s="21"/>
-      <c r="I23" s="57"/>
-      <c r="J23" s="57"/>
-      <c r="K23" s="57"/>
-      <c r="L23" s="53"/>
-      <c r="M23" s="53"/>
-      <c r="N23" s="53"/>
-      <c r="O23" s="53"/>
-      <c r="P23" s="53"/>
-      <c r="Q23" s="57"/>
-      <c r="R23" s="57"/>
-      <c r="S23" s="57"/>
+      <c r="I23" s="56"/>
+      <c r="J23" s="56"/>
+      <c r="K23" s="56"/>
+      <c r="L23" s="52"/>
+      <c r="M23" s="52"/>
+      <c r="N23" s="52"/>
+      <c r="O23" s="52"/>
+      <c r="P23" s="52"/>
+      <c r="Q23" s="56"/>
+      <c r="R23" s="56"/>
+      <c r="S23" s="56"/>
     </row>
     <row r="24" spans="1:19" ht="27" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A24" s="44" t="s">
+      <c r="A24" s="43" t="s">
         <v>21</v>
       </c>
       <c r="B24" s="23" t="s">
@@ -1986,20 +1977,20 @@
       <c r="F24" s="21"/>
       <c r="G24" s="21"/>
       <c r="H24" s="21"/>
-      <c r="I24" s="57"/>
-      <c r="J24" s="57"/>
-      <c r="K24" s="57"/>
-      <c r="L24" s="54"/>
-      <c r="M24" s="54"/>
-      <c r="N24" s="54"/>
-      <c r="O24" s="54"/>
-      <c r="P24" s="54"/>
-      <c r="Q24" s="57"/>
-      <c r="R24" s="57"/>
-      <c r="S24" s="57"/>
+      <c r="I24" s="56"/>
+      <c r="J24" s="56"/>
+      <c r="K24" s="56"/>
+      <c r="L24" s="53"/>
+      <c r="M24" s="53"/>
+      <c r="N24" s="53"/>
+      <c r="O24" s="53"/>
+      <c r="P24" s="53"/>
+      <c r="Q24" s="56"/>
+      <c r="R24" s="56"/>
+      <c r="S24" s="56"/>
     </row>
     <row r="25" spans="1:19" ht="22" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A25" s="45" t="str">
+      <c r="A25" s="44" t="str">
         <f>F13</f>
         <v>Non</v>
       </c>
@@ -2007,71 +1998,71 @@
       <c r="C25" s="11"/>
       <c r="D25" s="11"/>
       <c r="E25" s="11"/>
-      <c r="I25" s="57"/>
-      <c r="J25" s="57"/>
-      <c r="K25" s="57"/>
-      <c r="L25" s="57"/>
-      <c r="M25" s="59"/>
-      <c r="N25" s="60"/>
-      <c r="O25" s="57"/>
-      <c r="P25" s="57"/>
-      <c r="Q25" s="57"/>
-      <c r="R25" s="57"/>
-      <c r="S25" s="57"/>
+      <c r="I25" s="56"/>
+      <c r="J25" s="56"/>
+      <c r="K25" s="56"/>
+      <c r="L25" s="56"/>
+      <c r="M25" s="58"/>
+      <c r="N25" s="59"/>
+      <c r="O25" s="56"/>
+      <c r="P25" s="56"/>
+      <c r="Q25" s="56"/>
+      <c r="R25" s="56"/>
+      <c r="S25" s="56"/>
     </row>
     <row r="26" spans="1:19" ht="22" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A26"/>
-      <c r="I26" s="57"/>
-      <c r="J26" s="57"/>
-      <c r="K26" s="57"/>
-      <c r="L26" s="57"/>
-      <c r="M26" s="57"/>
-      <c r="N26" s="57"/>
-      <c r="O26" s="57"/>
-      <c r="P26" s="57"/>
-      <c r="Q26" s="57"/>
-      <c r="R26" s="57"/>
-      <c r="S26" s="57"/>
+      <c r="I26" s="56"/>
+      <c r="J26" s="56"/>
+      <c r="K26" s="56"/>
+      <c r="L26" s="56"/>
+      <c r="M26" s="56"/>
+      <c r="N26" s="56"/>
+      <c r="O26" s="56"/>
+      <c r="P26" s="56"/>
+      <c r="Q26" s="56"/>
+      <c r="R26" s="56"/>
+      <c r="S26" s="56"/>
     </row>
     <row r="27" spans="1:19" ht="22" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A27"/>
-      <c r="I27" s="57"/>
-      <c r="J27" s="57"/>
-      <c r="K27" s="57"/>
-      <c r="L27" s="58"/>
-      <c r="M27" s="57"/>
-      <c r="N27" s="57"/>
-      <c r="O27" s="57"/>
-      <c r="P27" s="57"/>
-      <c r="Q27" s="57"/>
-      <c r="R27" s="57"/>
-      <c r="S27" s="57"/>
+      <c r="I27" s="56"/>
+      <c r="J27" s="56"/>
+      <c r="K27" s="56"/>
+      <c r="L27" s="57"/>
+      <c r="M27" s="56"/>
+      <c r="N27" s="56"/>
+      <c r="O27" s="56"/>
+      <c r="P27" s="56"/>
+      <c r="Q27" s="56"/>
+      <c r="R27" s="56"/>
+      <c r="S27" s="56"/>
     </row>
     <row r="28" spans="1:19" ht="22" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A28" s="82" t="s">
+      <c r="A28" s="81" t="s">
         <v>20</v>
       </c>
-      <c r="B28" s="80"/>
-      <c r="C28" s="80"/>
-      <c r="D28" s="80"/>
-      <c r="E28" s="80"/>
-      <c r="F28" s="81"/>
+      <c r="B28" s="79"/>
+      <c r="C28" s="79"/>
+      <c r="D28" s="79"/>
+      <c r="E28" s="79"/>
+      <c r="F28" s="80"/>
       <c r="G28" s="21"/>
       <c r="H28" s="21"/>
-      <c r="I28" s="57"/>
-      <c r="J28" s="57"/>
-      <c r="K28" s="57"/>
-      <c r="L28" s="53"/>
-      <c r="M28" s="53"/>
-      <c r="N28" s="53"/>
-      <c r="O28" s="53"/>
-      <c r="P28" s="53"/>
-      <c r="Q28" s="53"/>
-      <c r="R28" s="57"/>
-      <c r="S28" s="57"/>
+      <c r="I28" s="56"/>
+      <c r="J28" s="56"/>
+      <c r="K28" s="56"/>
+      <c r="L28" s="52"/>
+      <c r="M28" s="52"/>
+      <c r="N28" s="52"/>
+      <c r="O28" s="52"/>
+      <c r="P28" s="52"/>
+      <c r="Q28" s="52"/>
+      <c r="R28" s="56"/>
+      <c r="S28" s="56"/>
     </row>
     <row r="29" spans="1:19" ht="36" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A29" s="46" t="s">
+      <c r="A29" s="45" t="s">
         <v>20</v>
       </c>
       <c r="B29" s="24" t="s">
@@ -2091,20 +2082,20 @@
       </c>
       <c r="G29" s="21"/>
       <c r="H29" s="21"/>
-      <c r="I29" s="57"/>
-      <c r="J29" s="57"/>
-      <c r="K29" s="57"/>
-      <c r="L29" s="54"/>
-      <c r="M29" s="55"/>
-      <c r="N29" s="56"/>
-      <c r="O29" s="54"/>
-      <c r="P29" s="54"/>
-      <c r="Q29" s="54"/>
-      <c r="R29" s="57"/>
-      <c r="S29" s="57"/>
+      <c r="I29" s="56"/>
+      <c r="J29" s="56"/>
+      <c r="K29" s="56"/>
+      <c r="L29" s="53"/>
+      <c r="M29" s="54"/>
+      <c r="N29" s="55"/>
+      <c r="O29" s="53"/>
+      <c r="P29" s="53"/>
+      <c r="Q29" s="53"/>
+      <c r="R29" s="56"/>
+      <c r="S29" s="56"/>
     </row>
     <row r="30" spans="1:19" ht="22" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A30" s="45" t="str">
+      <c r="A30" s="44" t="str">
         <f>D13</f>
         <v>Non</v>
       </c>
@@ -2115,71 +2106,71 @@
       <c r="F30" s="11"/>
       <c r="G30" s="21"/>
       <c r="H30" s="21"/>
-      <c r="I30" s="57"/>
-      <c r="J30" s="57"/>
-      <c r="K30" s="57"/>
-      <c r="L30" s="57"/>
-      <c r="M30" s="57"/>
-      <c r="N30" s="57"/>
-      <c r="O30" s="57"/>
-      <c r="P30" s="57"/>
-      <c r="Q30" s="57"/>
-      <c r="R30" s="57"/>
-      <c r="S30" s="57"/>
+      <c r="I30" s="56"/>
+      <c r="J30" s="56"/>
+      <c r="K30" s="56"/>
+      <c r="L30" s="56"/>
+      <c r="M30" s="56"/>
+      <c r="N30" s="56"/>
+      <c r="O30" s="56"/>
+      <c r="P30" s="56"/>
+      <c r="Q30" s="56"/>
+      <c r="R30" s="56"/>
+      <c r="S30" s="56"/>
     </row>
     <row r="31" spans="1:19" ht="22" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A31"/>
-      <c r="I31" s="57"/>
-      <c r="J31" s="57"/>
-      <c r="K31" s="57"/>
-      <c r="L31" s="57"/>
-      <c r="M31" s="57"/>
-      <c r="N31" s="57"/>
-      <c r="O31" s="57"/>
-      <c r="P31" s="57"/>
-      <c r="Q31" s="57"/>
-      <c r="R31" s="57"/>
-      <c r="S31" s="57"/>
+      <c r="I31" s="56"/>
+      <c r="J31" s="56"/>
+      <c r="K31" s="56"/>
+      <c r="L31" s="56"/>
+      <c r="M31" s="56"/>
+      <c r="N31" s="56"/>
+      <c r="O31" s="56"/>
+      <c r="P31" s="56"/>
+      <c r="Q31" s="56"/>
+      <c r="R31" s="56"/>
+      <c r="S31" s="56"/>
     </row>
     <row r="32" spans="1:19" ht="22" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A32"/>
-      <c r="I32" s="57"/>
-      <c r="J32" s="57"/>
-      <c r="K32" s="57"/>
-      <c r="L32" s="58"/>
-      <c r="M32" s="57"/>
-      <c r="N32" s="57"/>
-      <c r="O32" s="57"/>
-      <c r="P32" s="57"/>
-      <c r="Q32" s="57"/>
-      <c r="R32" s="57"/>
-      <c r="S32" s="57"/>
+      <c r="I32" s="56"/>
+      <c r="J32" s="56"/>
+      <c r="K32" s="56"/>
+      <c r="L32" s="57"/>
+      <c r="M32" s="56"/>
+      <c r="N32" s="56"/>
+      <c r="O32" s="56"/>
+      <c r="P32" s="56"/>
+      <c r="Q32" s="56"/>
+      <c r="R32" s="56"/>
+      <c r="S32" s="56"/>
     </row>
     <row r="33" spans="1:23" ht="22" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A33" s="91" t="s">
+      <c r="A33" s="90" t="s">
         <v>43</v>
       </c>
-      <c r="B33" s="89"/>
-      <c r="C33" s="89"/>
-      <c r="D33" s="89"/>
-      <c r="E33" s="89"/>
-      <c r="F33" s="89"/>
-      <c r="G33" s="89"/>
-      <c r="H33" s="90"/>
-      <c r="I33" s="57"/>
-      <c r="J33" s="57"/>
-      <c r="K33" s="57"/>
-      <c r="L33" s="53"/>
-      <c r="M33" s="53"/>
-      <c r="N33" s="53"/>
-      <c r="O33" s="53"/>
-      <c r="P33" s="53"/>
-      <c r="Q33" s="53"/>
-      <c r="R33" s="53"/>
-      <c r="S33" s="53"/>
+      <c r="B33" s="88"/>
+      <c r="C33" s="88"/>
+      <c r="D33" s="88"/>
+      <c r="E33" s="88"/>
+      <c r="F33" s="88"/>
+      <c r="G33" s="88"/>
+      <c r="H33" s="89"/>
+      <c r="I33" s="56"/>
+      <c r="J33" s="56"/>
+      <c r="K33" s="56"/>
+      <c r="L33" s="52"/>
+      <c r="M33" s="52"/>
+      <c r="N33" s="52"/>
+      <c r="O33" s="52"/>
+      <c r="P33" s="52"/>
+      <c r="Q33" s="52"/>
+      <c r="R33" s="52"/>
+      <c r="S33" s="52"/>
     </row>
     <row r="34" spans="1:23" ht="26" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A34" s="47" t="s">
+      <c r="A34" s="46" t="s">
         <v>22</v>
       </c>
       <c r="B34" s="3" t="s">
@@ -2203,111 +2194,111 @@
       <c r="H34" s="6" t="s">
         <v>48</v>
       </c>
-      <c r="I34" s="57"/>
-      <c r="J34" s="57"/>
-      <c r="K34" s="57"/>
-      <c r="L34" s="54"/>
-      <c r="M34" s="54"/>
-      <c r="N34" s="54"/>
-      <c r="O34" s="54"/>
-      <c r="P34" s="54"/>
-      <c r="Q34" s="54"/>
-      <c r="R34" s="54"/>
-      <c r="S34" s="54"/>
+      <c r="I34" s="56"/>
+      <c r="J34" s="56"/>
+      <c r="K34" s="56"/>
+      <c r="L34" s="53"/>
+      <c r="M34" s="53"/>
+      <c r="N34" s="53"/>
+      <c r="O34" s="53"/>
+      <c r="P34" s="53"/>
+      <c r="Q34" s="53"/>
+      <c r="R34" s="53"/>
+      <c r="S34" s="53"/>
     </row>
     <row r="35" spans="1:23" ht="22" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A35" s="48" t="str">
+      <c r="A35" s="47" t="str">
         <f>H13</f>
         <v>Non</v>
       </c>
       <c r="B35" s="2"/>
-      <c r="C35" s="48" t="str">
+      <c r="C35" s="47" t="str">
         <f>B14</f>
         <v>Non</v>
       </c>
       <c r="D35" s="2"/>
-      <c r="E35" s="48" t="str">
+      <c r="E35" s="47" t="str">
         <f>D14</f>
         <v>Non</v>
       </c>
       <c r="F35" s="2"/>
-      <c r="G35" s="48" t="str">
+      <c r="G35" s="47" t="str">
         <f>F14</f>
         <v>Non</v>
       </c>
       <c r="H35" s="2"/>
-      <c r="I35" s="57"/>
-      <c r="J35" s="57"/>
-      <c r="K35" s="57"/>
-      <c r="L35" s="57"/>
-      <c r="M35" s="57"/>
-      <c r="N35" s="59"/>
-      <c r="O35" s="60"/>
-      <c r="P35" s="57"/>
-      <c r="Q35" s="57"/>
-      <c r="R35" s="57"/>
-      <c r="S35" s="57"/>
+      <c r="I35" s="56"/>
+      <c r="J35" s="56"/>
+      <c r="K35" s="56"/>
+      <c r="L35" s="56"/>
+      <c r="M35" s="56"/>
+      <c r="N35" s="58"/>
+      <c r="O35" s="59"/>
+      <c r="P35" s="56"/>
+      <c r="Q35" s="56"/>
+      <c r="R35" s="56"/>
+      <c r="S35" s="56"/>
     </row>
     <row r="36" spans="1:23" ht="22" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A36"/>
-      <c r="I36" s="57"/>
-      <c r="J36" s="57"/>
-      <c r="K36" s="57"/>
-      <c r="L36" s="57"/>
-      <c r="M36" s="57"/>
-      <c r="N36" s="57"/>
-      <c r="O36" s="57"/>
-      <c r="P36" s="57"/>
-      <c r="Q36" s="57"/>
-      <c r="R36" s="57"/>
-      <c r="S36" s="57"/>
+      <c r="I36" s="56"/>
+      <c r="J36" s="56"/>
+      <c r="K36" s="56"/>
+      <c r="L36" s="56"/>
+      <c r="M36" s="56"/>
+      <c r="N36" s="56"/>
+      <c r="O36" s="56"/>
+      <c r="P36" s="56"/>
+      <c r="Q36" s="56"/>
+      <c r="R36" s="56"/>
+      <c r="S36" s="56"/>
     </row>
     <row r="37" spans="1:23" ht="22" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A37"/>
-      <c r="I37" s="57"/>
-      <c r="J37" s="57"/>
-      <c r="K37" s="57"/>
-      <c r="L37" s="58"/>
-      <c r="M37" s="57"/>
-      <c r="N37" s="57"/>
-      <c r="O37" s="57"/>
-      <c r="P37" s="57"/>
-      <c r="Q37" s="57"/>
-      <c r="R37" s="57"/>
-      <c r="S37" s="57"/>
+      <c r="I37" s="56"/>
+      <c r="J37" s="56"/>
+      <c r="K37" s="56"/>
+      <c r="L37" s="57"/>
+      <c r="M37" s="56"/>
+      <c r="N37" s="56"/>
+      <c r="O37" s="56"/>
+      <c r="P37" s="56"/>
+      <c r="Q37" s="56"/>
+      <c r="R37" s="56"/>
+      <c r="S37" s="56"/>
     </row>
     <row r="38" spans="1:23" ht="22" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A38" s="83" t="s">
+      <c r="A38" s="82" t="s">
         <v>18</v>
       </c>
-      <c r="B38" s="80"/>
-      <c r="C38" s="80"/>
-      <c r="D38" s="80"/>
-      <c r="E38" s="81"/>
+      <c r="B38" s="79"/>
+      <c r="C38" s="79"/>
+      <c r="D38" s="79"/>
+      <c r="E38" s="80"/>
       <c r="F38" s="21"/>
       <c r="G38" s="21"/>
       <c r="H38" s="21"/>
-      <c r="I38" s="57"/>
-      <c r="J38" s="57"/>
-      <c r="K38" s="57"/>
-      <c r="L38" s="53"/>
-      <c r="M38" s="53"/>
-      <c r="N38" s="53"/>
-      <c r="O38" s="53"/>
-      <c r="P38" s="53"/>
-      <c r="Q38" s="57"/>
-      <c r="R38" s="57"/>
-      <c r="S38" s="57"/>
+      <c r="I38" s="56"/>
+      <c r="J38" s="56"/>
+      <c r="K38" s="56"/>
+      <c r="L38" s="52"/>
+      <c r="M38" s="52"/>
+      <c r="N38" s="52"/>
+      <c r="O38" s="52"/>
+      <c r="P38" s="52"/>
+      <c r="Q38" s="56"/>
+      <c r="R38" s="56"/>
+      <c r="S38" s="56"/>
     </row>
     <row r="39" spans="1:23" ht="22" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A39" s="49" t="s">
+      <c r="A39" s="48" t="s">
         <v>18</v>
       </c>
-      <c r="B39" s="49" t="s">
-        <v>74</v>
-      </c>
-      <c r="C39" s="49" t="s">
-        <v>75</v>
+      <c r="B39" s="48" t="s">
+        <v>67</v>
+      </c>
+      <c r="C39" s="48" t="s">
+        <v>68</v>
       </c>
       <c r="D39" s="26" t="s">
         <v>50</v>
@@ -2321,165 +2312,155 @@
       <c r="G39" s="26" t="s">
         <v>49</v>
       </c>
-      <c r="I39" s="57"/>
-      <c r="J39" s="57"/>
-      <c r="K39" s="57"/>
-      <c r="L39" s="54"/>
-      <c r="M39" s="54"/>
-      <c r="N39" s="55"/>
-      <c r="O39" s="56"/>
-      <c r="P39" s="54"/>
-      <c r="Q39" s="57"/>
-      <c r="R39" s="57"/>
-      <c r="S39" s="57"/>
+      <c r="I39" s="56"/>
+      <c r="J39" s="56"/>
+      <c r="K39" s="56"/>
+      <c r="L39" s="53"/>
+      <c r="M39" s="53"/>
+      <c r="N39" s="54"/>
+      <c r="O39" s="55"/>
+      <c r="P39" s="53"/>
+      <c r="Q39" s="56"/>
+      <c r="R39" s="56"/>
+      <c r="S39" s="56"/>
     </row>
     <row r="40" spans="1:23" ht="22" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A40" s="45" t="str">
+      <c r="A40" s="44" t="str">
         <f>B13</f>
         <v>Non</v>
       </c>
-      <c r="B40" s="73"/>
-      <c r="C40" s="73"/>
+      <c r="B40" s="72"/>
+      <c r="C40" s="72"/>
       <c r="D40" s="25"/>
       <c r="E40" s="13"/>
       <c r="F40" s="11"/>
-      <c r="G40" s="96" t="str">
+      <c r="G40" s="75" t="str">
         <f>IF(OR(B40="",C40="",D40="",E40=""),"",UPPER(LEFT(B40,1))&amp;UPPER(MID(B40,FIND(" ",B40&amp;" ")+1,1))&amp;UPPER(LEFT(C40,1))&amp;UPPER(MID(C40,FIND(" ",C40&amp;" ")+1,1))&amp;"_"&amp;TEXT(D40,"aaaammjj")&amp;"_"&amp;TEXT(E40,"hh\hmm"))</f>
         <v/>
       </c>
-      <c r="I40" s="57"/>
-      <c r="J40" s="57"/>
-      <c r="K40" s="57"/>
-      <c r="L40" s="57"/>
-      <c r="M40" s="57"/>
-      <c r="N40" s="57"/>
-      <c r="O40" s="57"/>
-      <c r="P40" s="57"/>
-      <c r="Q40" s="57"/>
-      <c r="R40" s="57"/>
-      <c r="S40" s="57"/>
+      <c r="I40" s="56"/>
+      <c r="J40" s="56"/>
+      <c r="K40" s="56"/>
+      <c r="L40" s="56"/>
+      <c r="M40" s="56"/>
+      <c r="N40" s="56"/>
+      <c r="O40" s="56"/>
+      <c r="P40" s="56"/>
+      <c r="Q40" s="56"/>
+      <c r="R40" s="56"/>
+      <c r="S40" s="56"/>
     </row>
     <row r="41" spans="1:23" ht="22" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A41"/>
       <c r="F41" s="21"/>
       <c r="G41" s="21"/>
       <c r="H41" s="21"/>
-      <c r="I41" s="57"/>
-      <c r="J41" s="57"/>
-      <c r="K41" s="57"/>
-      <c r="L41" s="57"/>
-      <c r="M41" s="57"/>
-      <c r="N41" s="57"/>
-      <c r="O41" s="57"/>
-      <c r="P41" s="57"/>
-      <c r="Q41" s="57"/>
-      <c r="R41" s="61"/>
+      <c r="I41" s="56"/>
+      <c r="J41" s="56"/>
+      <c r="K41" s="56"/>
+      <c r="L41" s="56"/>
+      <c r="M41" s="56"/>
+      <c r="N41" s="56"/>
+      <c r="O41" s="56"/>
+      <c r="P41" s="56"/>
+      <c r="Q41" s="56"/>
+      <c r="R41" s="60"/>
     </row>
     <row r="42" spans="1:23" ht="22" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A42"/>
-      <c r="I42" s="57"/>
-      <c r="J42" s="57"/>
-      <c r="K42" s="57"/>
-      <c r="L42" s="58"/>
-      <c r="M42" s="57"/>
-      <c r="N42" s="57"/>
-      <c r="O42" s="57"/>
-      <c r="P42" s="57"/>
-      <c r="Q42" s="57"/>
-      <c r="R42" s="62"/>
-      <c r="S42" s="62"/>
-      <c r="T42" s="62"/>
-      <c r="U42" s="62"/>
-      <c r="V42" s="62"/>
-      <c r="W42" s="62"/>
+      <c r="I42" s="56"/>
+      <c r="J42" s="56"/>
+      <c r="K42" s="56"/>
+      <c r="L42" s="57"/>
+      <c r="M42" s="56"/>
+      <c r="N42" s="56"/>
+      <c r="O42" s="56"/>
+      <c r="P42" s="56"/>
+      <c r="Q42" s="56"/>
+      <c r="R42" s="61"/>
+      <c r="S42" s="61"/>
+      <c r="T42" s="61"/>
+      <c r="U42" s="61"/>
+      <c r="V42" s="61"/>
+      <c r="W42" s="61"/>
     </row>
     <row r="43" spans="1:23" ht="22" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A43" s="79" t="s">
-        <v>53</v>
-      </c>
-      <c r="B43" s="80"/>
-      <c r="C43" s="80"/>
-      <c r="D43" s="80"/>
-      <c r="E43" s="80"/>
-      <c r="F43" s="81"/>
+      <c r="A43" s="96" t="s">
+        <v>69</v>
+      </c>
+      <c r="B43" s="93"/>
+      <c r="C43" s="93"/>
+      <c r="D43" s="93"/>
+      <c r="E43" s="93"/>
+      <c r="F43" s="93"/>
       <c r="G43" s="21"/>
       <c r="H43" s="21"/>
-      <c r="I43" s="57"/>
-      <c r="J43" s="57"/>
-      <c r="K43" s="57"/>
-      <c r="L43" s="53"/>
-      <c r="M43" s="53"/>
-      <c r="N43" s="53"/>
-      <c r="O43" s="53"/>
-      <c r="P43" s="53"/>
-      <c r="Q43" s="53"/>
-      <c r="R43" s="57"/>
-      <c r="S43" s="57"/>
+      <c r="I43" s="56"/>
+      <c r="J43" s="56"/>
+      <c r="K43" s="56"/>
+      <c r="L43" s="52"/>
+      <c r="M43" s="52"/>
+      <c r="N43" s="52"/>
+      <c r="O43" s="52"/>
+      <c r="P43" s="52"/>
+      <c r="Q43" s="52"/>
+      <c r="R43" s="56"/>
+      <c r="S43" s="56"/>
     </row>
     <row r="44" spans="1:23" ht="34" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A44" s="74" t="s">
-        <v>54</v>
-      </c>
-      <c r="B44" s="75" t="s">
-        <v>55</v>
-      </c>
-      <c r="C44" s="75" t="s">
-        <v>56</v>
-      </c>
-      <c r="D44" s="75" t="s">
-        <v>57</v>
-      </c>
-      <c r="E44" s="75" t="s">
-        <v>58</v>
-      </c>
-      <c r="F44" s="75" t="s">
-        <v>59</v>
-      </c>
-      <c r="I44" s="57"/>
-      <c r="J44" s="57"/>
-      <c r="K44" s="57"/>
-      <c r="L44" s="54"/>
-      <c r="M44" s="54"/>
-      <c r="N44" s="54"/>
-      <c r="O44" s="54"/>
-      <c r="P44" s="54"/>
-      <c r="Q44" s="54"/>
-      <c r="R44" s="57"/>
-      <c r="S44" s="57"/>
-    </row>
-    <row r="45" spans="1:23" ht="22" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A45" s="43"/>
-      <c r="B45" s="11"/>
-      <c r="C45" s="11"/>
-      <c r="D45" s="11"/>
-      <c r="E45" s="11"/>
-      <c r="F45" s="11"/>
+      <c r="A44" s="97" t="s">
+        <v>70</v>
+      </c>
+      <c r="B44" s="94"/>
+      <c r="C44" s="94"/>
+      <c r="D44" s="94"/>
+      <c r="E44" s="94"/>
+      <c r="F44" s="94"/>
+      <c r="I44" s="56"/>
+      <c r="J44" s="56"/>
+      <c r="K44" s="56"/>
+      <c r="L44" s="53"/>
+      <c r="M44" s="53"/>
+      <c r="N44" s="53"/>
+      <c r="O44" s="53"/>
+      <c r="P44" s="53"/>
+      <c r="Q44" s="53"/>
+      <c r="R44" s="56"/>
+      <c r="S44" s="56"/>
+    </row>
+    <row r="45" spans="1:23" ht="22" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A45" s="98"/>
+      <c r="B45" s="95"/>
+      <c r="C45" s="95"/>
+      <c r="D45" s="95"/>
+      <c r="E45" s="95"/>
+      <c r="F45" s="95"/>
       <c r="G45" s="21"/>
-      <c r="I45" s="57"/>
-      <c r="J45" s="57"/>
-      <c r="K45" s="57"/>
-      <c r="L45" s="57"/>
-      <c r="M45" s="57"/>
-      <c r="N45" s="57"/>
-      <c r="O45" s="57"/>
-      <c r="P45" s="57"/>
-      <c r="Q45" s="57"/>
-      <c r="R45" s="57"/>
-      <c r="S45" s="57"/>
+      <c r="I45" s="56"/>
+      <c r="J45" s="56"/>
+      <c r="K45" s="56"/>
+      <c r="L45" s="56"/>
+      <c r="M45" s="56"/>
+      <c r="N45" s="56"/>
+      <c r="O45" s="56"/>
+      <c r="P45" s="56"/>
+      <c r="Q45" s="56"/>
+      <c r="R45" s="56"/>
+      <c r="S45" s="56"/>
     </row>
     <row r="46" spans="1:23" ht="22" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A46"/>
-      <c r="I46" s="57"/>
-      <c r="J46" s="57"/>
-      <c r="K46" s="57"/>
-      <c r="L46" s="57"/>
-      <c r="M46" s="57"/>
-      <c r="N46" s="57"/>
-      <c r="O46" s="57"/>
-      <c r="P46" s="57"/>
-      <c r="Q46" s="57"/>
-      <c r="R46" s="57"/>
-      <c r="S46" s="57"/>
+      <c r="I46" s="56"/>
+      <c r="J46" s="56"/>
+      <c r="K46" s="56"/>
+      <c r="L46" s="56"/>
+      <c r="M46" s="56"/>
+      <c r="N46" s="56"/>
+      <c r="O46" s="56"/>
+      <c r="P46" s="56"/>
+      <c r="Q46" s="56"/>
+      <c r="R46" s="56"/>
+      <c r="S46" s="56"/>
     </row>
     <row r="47" spans="1:23" ht="22" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A47" s="41"/>
@@ -2490,11 +2471,11 @@
       <c r="F47" s="21"/>
       <c r="G47" s="21"/>
       <c r="H47" s="21"/>
-      <c r="L47" s="53"/>
+      <c r="L47" s="52"/>
     </row>
     <row r="48" spans="1:23" ht="22" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A48" s="84" t="s">
-        <v>60</v>
+      <c r="A48" s="83" t="s">
+        <v>53</v>
       </c>
       <c r="B48" s="21"/>
       <c r="C48" s="21"/>
@@ -2503,11 +2484,11 @@
       <c r="F48" s="21"/>
       <c r="G48" s="21"/>
       <c r="H48" s="21"/>
-      <c r="L48" s="53"/>
+      <c r="L48" s="52"/>
     </row>
     <row r="49" spans="1:12" ht="22" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A49" s="50" t="s">
-        <v>61</v>
+      <c r="A49" s="49" t="s">
+        <v>54</v>
       </c>
       <c r="B49" s="21"/>
       <c r="C49" s="21"/>
@@ -2516,11 +2497,11 @@
       <c r="F49" s="21"/>
       <c r="G49" s="21"/>
       <c r="H49" s="21"/>
-      <c r="L49" s="54"/>
+      <c r="L49" s="53"/>
     </row>
     <row r="50" spans="1:12" ht="22" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A50" s="11" t="s">
-        <v>73</v>
+        <v>66</v>
       </c>
       <c r="B50" s="21"/>
       <c r="C50" s="21"/>
@@ -2531,10 +2512,8 @@
       <c r="H50" s="21"/>
     </row>
   </sheetData>
-  <sheetProtection sheet="1"/>
-  <mergeCells count="10">
+  <mergeCells count="9">
     <mergeCell ref="A1:H1"/>
-    <mergeCell ref="A43:F43"/>
     <mergeCell ref="A28:F28"/>
     <mergeCell ref="A38:E38"/>
     <mergeCell ref="A48"/>
@@ -2544,7 +2523,7 @@
     <mergeCell ref="A23:E23"/>
     <mergeCell ref="A18:F18"/>
   </mergeCells>
-  <dataValidations count="21">
+  <dataValidations count="20">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Météo invalide" error="Choisissez une météo dans la liste." promptTitle="Météo" prompt="Choisir une condition météo" sqref="A16 L15 A20" xr:uid="{00000000-0002-0000-0000-000000000000}">
       <formula1>"Ensoleillé,Nuageux,Couvert,Petite pluie,Pluie forte,Orage"</formula1>
     </dataValidation>
@@ -2597,10 +2576,9 @@
     <dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Nom du prélèvement" prompt="Se remplit automatiquement lorsque les informations générales seront remplies. Enregistrer le fichier sous ce nom." sqref="B3" xr:uid="{424D348A-D12B-8742-B0EB-C37623FAD8F4}">
       <formula1>TRUE</formula1>
     </dataValidation>
-    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Date" prompt="Saisir une date au format jj/mm/aaaa" sqref="B30" xr:uid="{A0AE77B4-9F2E-3A47-AAB7-800774FFD168}"/>
+    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Date" prompt="Saisir une date au format jj/mm/aaaa" sqref="B30 D40" xr:uid="{A0AE77B4-9F2E-3A47-AAB7-800774FFD168}"/>
     <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Heure" prompt="Saisir une heure au format hh:mm" sqref="F20 C30 E40" xr:uid="{ED9B56F9-3443-344C-A717-B6C0E25FEB49}"/>
     <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Température" prompt="en °C" sqref="B20:C20" xr:uid="{06DF3729-F159-3D41-AF3F-54E70FBFB3A9}"/>
-    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Date" prompt="Saisir une date au format jj/mm/aaaa" sqref="D40" xr:uid="{D1E12E3D-80DF-3740-A9E3-03BE02A08F1A}"/>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <extLst>
@@ -2630,47 +2608,47 @@
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>71</v>
+        <v>64</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>64</v>
+        <v>57</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>65</v>
+        <v>58</v>
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>63</v>
+        <v>56</v>
       </c>
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>66</v>
+        <v>59</v>
       </c>
     </row>
     <row r="7" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
-        <v>67</v>
+        <v>60</v>
       </c>
     </row>
     <row r="8" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
-        <v>68</v>
+        <v>61</v>
       </c>
     </row>
     <row r="9" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
-        <v>69</v>
+        <v>62</v>
       </c>
     </row>
     <row r="10" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
-        <v>70</v>
+        <v>63</v>
       </c>
     </row>
   </sheetData>

</xml_diff>